<commit_message>
actualizar tabla de contenidos
</commit_message>
<xml_diff>
--- a/docs/networks.xlsx
+++ b/docs/networks.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\networks\server-hacking\nssh-mj19\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041733AB-6407-471E-AB51-5ACE95CECC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE15FE3-039B-44E9-B17D-AECA8B59D015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{D01C2053-D11D-4E53-94C6-551C8782C843}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="6" xr2:uid="{D01C2053-D11D-4E53-94C6-551C8782C843}"/>
   </bookViews>
   <sheets>
     <sheet name="Cifrado" sheetId="4" r:id="rId1"/>
     <sheet name="Unidades" sheetId="3" r:id="rId2"/>
     <sheet name="Modelos" sheetId="5" r:id="rId3"/>
+    <sheet name="acceso" sheetId="6" r:id="rId4"/>
+    <sheet name="internet" sheetId="7" r:id="rId5"/>
+    <sheet name="transporte" sheetId="8" r:id="rId6"/>
+    <sheet name="aplicacion" sheetId="9" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="DESPLAZAMIENTO">Cifrado!$Z$4</definedName>
@@ -41,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="216">
   <si>
     <t>C</t>
   </si>
@@ -410,13 +414,296 @@
   </si>
   <si>
     <t>10GBaseTX - 100BaseCx - 10GBaseLX</t>
+  </si>
+  <si>
+    <t>ETHERNET</t>
+  </si>
+  <si>
+    <t>EJEMPLO</t>
+  </si>
+  <si>
+    <t>ARP</t>
+  </si>
+  <si>
+    <t>UNICAST</t>
+  </si>
+  <si>
+    <t>MULTICAST</t>
+  </si>
+  <si>
+    <t>BROADCAST</t>
+  </si>
+  <si>
+    <t>El Destinatario es un HOST</t>
+  </si>
+  <si>
+    <t>El Destinatario es un Grupo de HOSTS</t>
+  </si>
+  <si>
+    <t>Los Destinatarios son Todos los HOSTS</t>
+  </si>
+  <si>
+    <t>Capa 2</t>
+  </si>
+  <si>
+    <t>Capa 3</t>
+  </si>
+  <si>
+    <t>Modelo</t>
+  </si>
+  <si>
+    <t>Unicast</t>
+  </si>
+  <si>
+    <t>Multicast</t>
+  </si>
+  <si>
+    <t>Broadcast</t>
+  </si>
+  <si>
+    <t>192.168.0.1</t>
+  </si>
+  <si>
+    <t>0800.272D.E8B7</t>
+  </si>
+  <si>
+    <t>224.0.0.2</t>
+  </si>
+  <si>
+    <t>FFFF.FFFF.FFFF</t>
+  </si>
+  <si>
+    <t>DST MAC</t>
+  </si>
+  <si>
+    <t>SRC MAC</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>PAYLOAD</t>
+  </si>
+  <si>
+    <t>FCS</t>
+  </si>
+  <si>
+    <t>A051.50A1.6A12</t>
+  </si>
+  <si>
+    <t>0x806 (ARP)</t>
+  </si>
+  <si>
+    <t>SRC IP</t>
+  </si>
+  <si>
+    <t>TARGET IP</t>
+  </si>
+  <si>
+    <t>TARGET MAC</t>
+  </si>
+  <si>
+    <t>SOURCE IP</t>
+  </si>
+  <si>
+    <t>SOURCE MAC</t>
+  </si>
+  <si>
+    <t>VERSION</t>
+  </si>
+  <si>
+    <t>IPv4</t>
+  </si>
+  <si>
+    <t>192.168.0.2</t>
+  </si>
+  <si>
+    <t>0000.0000.0000</t>
+  </si>
+  <si>
+    <t>TTL</t>
+  </si>
+  <si>
+    <t>DST IP</t>
+  </si>
+  <si>
+    <t>CHECKSUM</t>
+  </si>
+  <si>
+    <t>TCP</t>
+  </si>
+  <si>
+    <t>SRC PORT</t>
+  </si>
+  <si>
+    <t>DST PORT</t>
+  </si>
+  <si>
+    <t>SEQ</t>
+  </si>
+  <si>
+    <t>ACK</t>
+  </si>
+  <si>
+    <t>WINDOW</t>
+  </si>
+  <si>
+    <t>PORTS</t>
+  </si>
+  <si>
+    <t>CONOCIDO</t>
+  </si>
+  <si>
+    <t>REGISTRADO</t>
+  </si>
+  <si>
+    <t>DINAMICO</t>
+  </si>
+  <si>
+    <t>INI</t>
+  </si>
+  <si>
+    <t>FIN</t>
+  </si>
+  <si>
+    <t>0800.0B07:0DB8</t>
+  </si>
+  <si>
+    <t>MENSAJE</t>
+  </si>
+  <si>
+    <t>DESCRIPCION</t>
+  </si>
+  <si>
+    <t>0180.c200.0000</t>
+  </si>
+  <si>
+    <t>0x0800 (IPv4)</t>
+  </si>
+  <si>
+    <t>0100 (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UDP </t>
+  </si>
+  <si>
+    <t>Clase</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>PUBLICO</t>
+  </si>
+  <si>
+    <t>PRIVADO</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>0.0.0.0</t>
+  </si>
+  <si>
+    <t>128.0.0.0</t>
+  </si>
+  <si>
+    <t>192.0.0.0</t>
+  </si>
+  <si>
+    <t>224.0.0.0</t>
+  </si>
+  <si>
+    <t>240.0.0.0</t>
+  </si>
+  <si>
+    <t>127.255.255.255</t>
+  </si>
+  <si>
+    <t>191.255.255.255</t>
+  </si>
+  <si>
+    <t>223.255.255.255</t>
+  </si>
+  <si>
+    <t>239.255.255.255</t>
+  </si>
+  <si>
+    <t>255.255.255.255</t>
+  </si>
+  <si>
+    <t>10.0.0.0</t>
+  </si>
+  <si>
+    <t>172.16.0.0</t>
+  </si>
+  <si>
+    <t>192.168.0.0</t>
+  </si>
+  <si>
+    <t>RESEARCH</t>
+  </si>
+  <si>
+    <t>10.255.255.255</t>
+  </si>
+  <si>
+    <t>172.31.255.255</t>
+  </si>
+  <si>
+    <t>192.168.255.255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIN </t>
+  </si>
+  <si>
+    <t>BIN</t>
+  </si>
+  <si>
+    <t>00000000</t>
+  </si>
+  <si>
+    <t>10000000</t>
+  </si>
+  <si>
+    <t>11000000</t>
+  </si>
+  <si>
+    <t>11100000</t>
+  </si>
+  <si>
+    <t>11110000</t>
+  </si>
+  <si>
+    <t>01111111</t>
+  </si>
+  <si>
+    <t>10111111</t>
+  </si>
+  <si>
+    <t>11011111</t>
+  </si>
+  <si>
+    <t>11101111</t>
+  </si>
+  <si>
+    <t>11111111</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -453,8 +740,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -488,6 +789,48 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor theme="4" tint="-0.499984740745262"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor theme="4" tint="-0.249977111117893"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor theme="3" tint="0.249977111117893"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor theme="9" tint="-0.249977111117893"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor theme="5" tint="-0.249977111117893"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFC00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -649,11 +992,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -738,52 +1082,295 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="1" builtinId="29"/>
+    <cellStyle name="Millares" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF9900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -793,6 +1380,94 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{8BD596F1-8187-48AD-A770-ECD0D83DD409}" name="Tabla5" displayName="Tabla5" ref="A1:B6" totalsRowShown="0">
+  <autoFilter ref="A1:B6" xr:uid="{8BD596F1-8187-48AD-A770-ECD0D83DD409}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{16412166-6806-49A6-8A76-2C57555AE578}" name="ETHERNET"/>
+    <tableColumn id="2" xr3:uid="{4059F672-4C51-4DBD-887A-E6C3AB5B42C4}" name="EJEMPLO" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7EFC7C69-423A-4037-823D-B3D1C6CE32AF}" name="Tabla6" displayName="Tabla6" ref="D1:E6" totalsRowShown="0">
+  <autoFilter ref="D1:E6" xr:uid="{7EFC7C69-423A-4037-823D-B3D1C6CE32AF}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{8F932B49-C9C7-4741-AE77-6700E1E04F7A}" name="ARP"/>
+    <tableColumn id="2" xr3:uid="{AA30F081-100A-4F91-A5D1-91ADC022F282}" name="EJEMPLO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9EC927FF-E91A-45E2-ABF7-94344CA4FD86}" name="Tabla58" displayName="Tabla58" ref="A8:B13" totalsRowShown="0">
+  <autoFilter ref="A8:B13" xr:uid="{9EC927FF-E91A-45E2-ABF7-94344CA4FD86}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{9FDDC075-BA29-4E23-8B93-0669E55677F6}" name="ETHERNET"/>
+    <tableColumn id="2" xr3:uid="{35A287F2-258E-4D1D-A0A0-84E3BE38046C}" name="EJEMPLO" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{1B209C23-92F8-4B29-8DE2-5F8BF2A75FBD}" name="Tabla611" displayName="Tabla611" ref="D8:E13" totalsRowShown="0">
+  <autoFilter ref="D8:E13" xr:uid="{1B209C23-92F8-4B29-8DE2-5F8BF2A75FBD}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{9CB76D8A-2370-4030-BB50-D5A772AF17D0}" name="ARP"/>
+    <tableColumn id="2" xr3:uid="{2D9C22FF-2977-46BD-96D7-302B01D80085}" name="EJEMPLO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{44F086F8-F65E-455D-A67A-8C950A8413AE}" name="Tabla4" displayName="Tabla4" ref="A1:B7" totalsRowShown="0">
+  <autoFilter ref="A1:B7" xr:uid="{44F086F8-F65E-455D-A67A-8C950A8413AE}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{FC9D1EB7-7AD0-40FF-AD53-F50391CFA555}" name="IPv4"/>
+    <tableColumn id="2" xr3:uid="{30CFA4BB-7536-4CC3-B3AB-8EA26AEA08CA}" name="EJEMPLO" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{743024AB-B1A3-465A-BED0-E7AD1A5BD48F}" name="Tabla2" displayName="Tabla2" ref="A1:B7" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="11">
+  <autoFilter ref="A1:B7" xr:uid="{743024AB-B1A3-465A-BED0-E7AD1A5BD48F}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{7CC5C3E3-99F7-406B-BE33-6498B71C96B5}" name="TCP" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{DFE11A21-5EAF-4D74-8E80-946C3D01C1E9}" name="EJEMPLO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{111471CA-6650-48C8-8EC8-4C882BF84B6D}" name="Tabla3" displayName="Tabla3" ref="D1:E5" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="8">
+  <autoFilter ref="D1:E5" xr:uid="{111471CA-6650-48C8-8EC8-4C882BF84B6D}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{D6C9935A-7A1F-4112-B3D6-F92843577E9E}" name="UDP "/>
+    <tableColumn id="2" xr3:uid="{0C921597-5962-46B5-A408-FAF1D8CFE85A}" name="EJEMPLO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C49B0AFB-4411-4BA3-9597-4305D7D964A7}" name="Tabla314" displayName="Tabla314" ref="D7:E11" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="0" tableBorderDxfId="1">
+  <autoFilter ref="D7:E11" xr:uid="{C49B0AFB-4411-4BA3-9597-4305D7D964A7}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{B6A9C988-3650-4A08-8C2D-DE663BBA1EBC}" name="UDP "/>
+    <tableColumn id="2" xr3:uid="{A846B633-9F69-4FA1-B3C6-4FB6EAE3A134}" name="EJEMPLO"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1116,34 +1791,34 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="4.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="34"/>
-      <c r="R1" s="34"/>
-      <c r="S1" s="34"/>
-      <c r="T1" s="34"/>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
-      <c r="W1" s="34"/>
-      <c r="X1" s="34"/>
-      <c r="Y1" s="34"/>
-      <c r="Z1" s="34"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="46"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1326,35 +2001,35 @@
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="37"/>
-      <c r="S4" s="38" t="s">
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="48"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="48"/>
+      <c r="P4" s="48"/>
+      <c r="Q4" s="48"/>
+      <c r="R4" s="49"/>
+      <c r="S4" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="T4" s="39"/>
-      <c r="U4" s="39"/>
-      <c r="V4" s="39"/>
-      <c r="W4" s="39"/>
-      <c r="X4" s="39"/>
-      <c r="Y4" s="40"/>
+      <c r="T4" s="51"/>
+      <c r="U4" s="51"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="51"/>
+      <c r="Y4" s="52"/>
       <c r="Z4" s="2">
         <v>4</v>
       </c>
@@ -1591,18 +2266,18 @@
       <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
       <c r="E3" s="10"/>
-      <c r="F3" s="33" t="s">
+      <c r="F3" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
@@ -1777,11 +2452,11 @@
         <v>53</v>
       </c>
       <c r="E11" s="10"/>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="33"/>
-      <c r="H11" s="33"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -1916,16 +2591,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF2CD719-EB61-4BC0-8AA0-D1D0CBFEE446}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.140625" customWidth="1"/>
-    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>98</v>
       </c>
@@ -1938,102 +2619,158 @@
       <c r="E1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G1" s="62" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1" s="73" t="s">
+        <v>175</v>
+      </c>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="55" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="57" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="55" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G2" s="63" t="s">
+        <v>126</v>
+      </c>
+      <c r="H2" s="70" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="42"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C3" s="55"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="55"/>
+      <c r="G3" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="H3" s="71" t="s">
+        <v>130</v>
+      </c>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="42"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C4" s="55"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="55"/>
+      <c r="G4" s="66" t="s">
+        <v>128</v>
+      </c>
+      <c r="H4" s="72" t="s">
+        <v>131</v>
+      </c>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="37" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="39" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G6" s="74" t="s">
+        <v>134</v>
+      </c>
+      <c r="H6" s="74" t="s">
+        <v>135</v>
+      </c>
+      <c r="I6" s="74" t="s">
+        <v>136</v>
+      </c>
+      <c r="J6" s="74" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="56" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G7" s="69" t="s">
+        <v>132</v>
+      </c>
+      <c r="H7" s="75" t="s">
+        <v>139</v>
+      </c>
+      <c r="I7" s="75" t="s">
+        <v>176</v>
+      </c>
+      <c r="J7" s="75" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="42" t="s">
         <v>106</v>
       </c>
       <c r="C8" s="43" t="s">
@@ -2042,10 +2779,22 @@
       <c r="D8" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="E8" s="42"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="41" t="s">
+      <c r="E8" s="56"/>
+      <c r="G8" s="76" t="s">
+        <v>133</v>
+      </c>
+      <c r="H8" s="77" t="s">
+        <v>138</v>
+      </c>
+      <c r="I8" s="77" t="s">
+        <v>140</v>
+      </c>
+      <c r="J8" s="78">
+        <v>255255255255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="32" t="s">
         <v>109</v>
       </c>
       <c r="E9" t="s">
@@ -2053,12 +2802,926 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="H1:J1"/>
     <mergeCell ref="E2:E4"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="C2:C4"/>
     <mergeCell ref="D2:D4"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="H4:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0636A6D-C6BF-4C55-BD89-4473DDA2952D}">
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="2.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="D4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" s="76" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>331F017E</v>
+      </c>
+      <c r="D6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" t="s">
+        <v>153</v>
+      </c>
+      <c r="E10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="D11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" t="s">
+        <v>151</v>
+      </c>
+      <c r="E12" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="76" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>95E82C30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="4">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0A9F5EE-A44D-4048-8F9E-918C91B2F299}">
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="15.5703125" style="44" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="82" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="10" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E1" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="81" t="s">
+        <v>185</v>
+      </c>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E2" s="82" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="44">
+        <v>128</v>
+      </c>
+      <c r="D3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E3" s="82" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="G3" s="84" t="s">
+        <v>192</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="I3" s="82" t="s">
+        <v>197</v>
+      </c>
+      <c r="K3" s="84" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E4" s="82" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="G4" s="84" t="s">
+        <v>193</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="I4" s="82" t="s">
+        <v>198</v>
+      </c>
+      <c r="K4" s="84" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="45">
+        <v>255255255255</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>189</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="G5" s="84" t="s">
+        <v>194</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="I5" s="82" t="s">
+        <v>199</v>
+      </c>
+      <c r="K5" s="84" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="82" t="s">
+        <v>190</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="G6" s="84" t="s">
+        <v>195</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="I6" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="J6" s="81"/>
+      <c r="K6" s="81"/>
+      <c r="L6" s="81"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="79" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>D8258CFE</v>
+      </c>
+      <c r="D7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="82" t="s">
+        <v>191</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="G7" s="84" t="s">
+        <v>196</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="I7" s="81" t="s">
+        <v>200</v>
+      </c>
+      <c r="J7" s="81"/>
+      <c r="K7" s="81"/>
+      <c r="L7" s="81"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E8" s="83">
+        <f>2^32</f>
+        <v>4294967296</v>
+      </c>
+      <c r="F8" s="83"/>
+      <c r="G8" s="83"/>
+      <c r="H8" s="83"/>
+      <c r="I8" s="83">
+        <f>2^32</f>
+        <v>4294967296</v>
+      </c>
+      <c r="J8" s="83"/>
+      <c r="K8" s="83"/>
+      <c r="L8" s="83"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="59" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="67" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="68">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="59" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12" s="67" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="60" t="s">
+        <v>159</v>
+      </c>
+      <c r="B13" s="80" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="59" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" s="67" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="79" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>66D08586</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="I8:L8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F965054-DFCE-48ED-9072-C1D7AD8FAEC1}">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="64" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="65" t="s">
+        <v>179</v>
+      </c>
+      <c r="E1" s="65" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="58" t="s">
+        <v>167</v>
+      </c>
+      <c r="H1" s="58" t="s">
+        <v>171</v>
+      </c>
+      <c r="I1" s="58" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="63">
+        <v>49810</v>
+      </c>
+      <c r="D2" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="E2" s="63">
+        <v>68</v>
+      </c>
+      <c r="G2" s="63" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="63">
+        <v>0</v>
+      </c>
+      <c r="I2" s="63">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" s="60">
+        <v>22</v>
+      </c>
+      <c r="D3" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="E3" s="60">
+        <v>67</v>
+      </c>
+      <c r="G3" s="60" t="s">
+        <v>169</v>
+      </c>
+      <c r="H3" s="60">
+        <v>1024</v>
+      </c>
+      <c r="I3" s="60">
+        <v>49151</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="59" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="59">
+        <v>0</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="59">
+        <v>65535</v>
+      </c>
+      <c r="G4" s="59" t="s">
+        <v>170</v>
+      </c>
+      <c r="H4" s="59">
+        <v>49152</v>
+      </c>
+      <c r="I4" s="59">
+        <v>65535</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="60">
+        <v>0</v>
+      </c>
+      <c r="D5" s="60" t="s">
+        <v>160</v>
+      </c>
+      <c r="E5" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>F5FCFD96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="59">
+        <v>65535</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>9272EBB7</v>
+      </c>
+      <c r="D7" s="65" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="65" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="E8" s="63">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
+        <v>161</v>
+      </c>
+      <c r="B9" s="58" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="E9" s="60">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" s="63">
+        <v>22</v>
+      </c>
+      <c r="D10" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="E10" s="59">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="60">
+        <v>49810</v>
+      </c>
+      <c r="D11" s="60" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>5D15AE6D</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="59" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12" s="59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" s="60">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="B14" s="59">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="61" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>189999A6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="58" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" s="58" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="63">
+        <v>49810</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" s="60">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="59" t="s">
+        <v>164</v>
+      </c>
+      <c r="B20" s="59">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B21" s="60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="B22" s="59">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B23" s="61" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>1F3E77C1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="58" t="s">
+        <v>161</v>
+      </c>
+      <c r="B25" s="58" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B26" s="63">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B27" s="60">
+        <v>49810</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="59" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" s="59">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B29" s="60">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="59">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="61" t="str">
+        <f ca="1">DEC2HEX((RAND()*2^32))</f>
+        <v>A7CAFF7E</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DEA4679-6A3B-48B4-A6B0-AA1541FF8CF5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
actualizar plantilla con ejemplos de umask
</commit_message>
<xml_diff>
--- a/docs/networks.xlsx
+++ b/docs/networks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EducacionIT\Documents\networks\server-hacking\nssh-mj19\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE15FE3-039B-44E9-B17D-AECA8B59D015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1671D3-0C52-4FE3-B218-519B2EABDE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="6" xr2:uid="{D01C2053-D11D-4E53-94C6-551C8782C843}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="7" xr2:uid="{D01C2053-D11D-4E53-94C6-551C8782C843}"/>
   </bookViews>
   <sheets>
     <sheet name="Cifrado" sheetId="4" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="internet" sheetId="7" r:id="rId5"/>
     <sheet name="transporte" sheetId="8" r:id="rId6"/>
     <sheet name="aplicacion" sheetId="9" r:id="rId7"/>
+    <sheet name="sistemas" sheetId="10" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="DESPLAZAMIENTO">Cifrado!$Z$4</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="257">
   <si>
     <t>C</t>
   </si>
@@ -693,6 +694,129 @@
   </si>
   <si>
     <t>11111111</t>
+  </si>
+  <si>
+    <t>DEC</t>
+  </si>
+  <si>
+    <t>HEX</t>
+  </si>
+  <si>
+    <t>OCT</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>000</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>--x</t>
+  </si>
+  <si>
+    <t>-w-</t>
+  </si>
+  <si>
+    <t>-wx</t>
+  </si>
+  <si>
+    <t>r--</t>
+  </si>
+  <si>
+    <t>r-x</t>
+  </si>
+  <si>
+    <t>rw-</t>
+  </si>
+  <si>
+    <t>rwx</t>
+  </si>
+  <si>
+    <t>Ninguno</t>
+  </si>
+  <si>
+    <t>Ejecucion</t>
+  </si>
+  <si>
+    <t>Escritura</t>
+  </si>
+  <si>
+    <t>Ejecutar y Escribir</t>
+  </si>
+  <si>
+    <t>Lectura</t>
+  </si>
+  <si>
+    <t>Leer y Ejecutar</t>
+  </si>
+  <si>
+    <t>Lectoescritura</t>
+  </si>
+  <si>
+    <t>Control Total</t>
+  </si>
+  <si>
+    <t>PERMISOS</t>
+  </si>
+  <si>
+    <t>ORDEN</t>
+  </si>
+  <si>
+    <t>Propietario</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Otros</t>
   </si>
 </sst>
 </file>
@@ -701,7 +825,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -997,7 +1121,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1124,6 +1248,42 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1151,6 +1311,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1160,69 +1323,22 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="1" builtinId="29"/>
@@ -1232,16 +1348,16 @@
   <dxfs count="12">
     <dxf>
       <border outline="0">
-        <bottom style="medium">
+        <top style="medium">
           <color theme="1"/>
-        </bottom>
+        </top>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="medium">
+        <bottom style="medium">
           <color theme="1"/>
-        </top>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1269,50 +1385,17 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <border outline="0">
         <bottom style="medium">
           <color theme="1"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color theme="1"/>
-        </top>
       </border>
     </dxf>
     <dxf>
@@ -1364,6 +1447,39 @@
         </top>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1387,7 +1503,7 @@
   <autoFilter ref="A1:B6" xr:uid="{8BD596F1-8187-48AD-A770-ECD0D83DD409}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{16412166-6806-49A6-8A76-2C57555AE578}" name="ETHERNET"/>
-    <tableColumn id="2" xr3:uid="{4059F672-4C51-4DBD-887A-E6C3AB5B42C4}" name="EJEMPLO" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{4059F672-4C51-4DBD-887A-E6C3AB5B42C4}" name="EJEMPLO" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1409,7 +1525,7 @@
   <autoFilter ref="A8:B13" xr:uid="{9EC927FF-E91A-45E2-ABF7-94344CA4FD86}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{9FDDC075-BA29-4E23-8B93-0669E55677F6}" name="ETHERNET"/>
-    <tableColumn id="2" xr3:uid="{35A287F2-258E-4D1D-A0A0-84E3BE38046C}" name="EJEMPLO" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{35A287F2-258E-4D1D-A0A0-84E3BE38046C}" name="EJEMPLO" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1431,17 +1547,17 @@
   <autoFilter ref="A1:B7" xr:uid="{44F086F8-F65E-455D-A67A-8C950A8413AE}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{FC9D1EB7-7AD0-40FF-AD53-F50391CFA555}" name="IPv4"/>
-    <tableColumn id="2" xr3:uid="{30CFA4BB-7536-4CC3-B3AB-8EA26AEA08CA}" name="EJEMPLO" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{30CFA4BB-7536-4CC3-B3AB-8EA26AEA08CA}" name="EJEMPLO" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{743024AB-B1A3-465A-BED0-E7AD1A5BD48F}" name="Tabla2" displayName="Tabla2" ref="A1:B7" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{743024AB-B1A3-465A-BED0-E7AD1A5BD48F}" name="Tabla2" displayName="Tabla2" ref="A1:B7" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
   <autoFilter ref="A1:B7" xr:uid="{743024AB-B1A3-465A-BED0-E7AD1A5BD48F}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CC5C3E3-99F7-406B-BE33-6498B71C96B5}" name="TCP" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{7CC5C3E3-99F7-406B-BE33-6498B71C96B5}" name="TCP" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{DFE11A21-5EAF-4D74-8E80-946C3D01C1E9}" name="EJEMPLO"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1449,7 +1565,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{111471CA-6650-48C8-8EC8-4C882BF84B6D}" name="Tabla3" displayName="Tabla3" ref="D1:E5" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{111471CA-6650-48C8-8EC8-4C882BF84B6D}" name="Tabla3" displayName="Tabla3" ref="D1:E5" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
   <autoFilter ref="D1:E5" xr:uid="{111471CA-6650-48C8-8EC8-4C882BF84B6D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D6C9935A-7A1F-4112-B3D6-F92843577E9E}" name="UDP "/>
@@ -1460,7 +1576,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C49B0AFB-4411-4BA3-9597-4305D7D964A7}" name="Tabla314" displayName="Tabla314" ref="D7:E11" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="0" tableBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C49B0AFB-4411-4BA3-9597-4305D7D964A7}" name="Tabla314" displayName="Tabla314" ref="D7:E11" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="D7:E11" xr:uid="{C49B0AFB-4411-4BA3-9597-4305D7D964A7}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{B6A9C988-3650-4A08-8C2D-DE663BBA1EBC}" name="UDP "/>
@@ -1791,34 +1907,34 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="4.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="46"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -2001,35 +2117,35 @@
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48"/>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="49"/>
-      <c r="S4" s="50" t="s">
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="T4" s="51"/>
-      <c r="U4" s="51"/>
-      <c r="V4" s="51"/>
-      <c r="W4" s="51"/>
-      <c r="X4" s="51"/>
-      <c r="Y4" s="52"/>
+      <c r="T4" s="67"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="68"/>
       <c r="Z4" s="2">
         <v>4</v>
       </c>
@@ -2266,18 +2382,18 @@
       <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
       <c r="E3" s="10"/>
-      <c r="F3" s="54" t="s">
+      <c r="F3" s="70" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
@@ -2452,11 +2568,11 @@
         <v>53</v>
       </c>
       <c r="E11" s="10"/>
-      <c r="F11" s="54" t="s">
+      <c r="F11" s="70" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
+      <c r="G11" s="70"/>
+      <c r="H11" s="70"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -2619,14 +2735,14 @@
       <c r="E1" t="s">
         <v>99</v>
       </c>
-      <c r="G1" s="62" t="s">
+      <c r="G1" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="H1" s="73" t="s">
+      <c r="H1" s="71" t="s">
         <v>175</v>
       </c>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -2635,23 +2751,23 @@
       <c r="B2" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="55" t="s">
+      <c r="C2" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="D2" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="55" t="s">
+      <c r="E2" s="72" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="63" t="s">
+      <c r="G2" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="H2" s="70" t="s">
+      <c r="H2" s="75" t="s">
         <v>129</v>
       </c>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -2660,17 +2776,17 @@
       <c r="B3" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="55"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="55"/>
-      <c r="G3" s="60" t="s">
+      <c r="C3" s="72"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="72"/>
+      <c r="G3" t="s">
         <v>127</v>
       </c>
-      <c r="H3" s="71" t="s">
+      <c r="H3" s="76" t="s">
         <v>130</v>
       </c>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
     </row>
     <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -2679,17 +2795,17 @@
       <c r="B4" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="55"/>
-      <c r="G4" s="66" t="s">
+      <c r="C4" s="72"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="72"/>
+      <c r="G4" s="51" t="s">
         <v>128</v>
       </c>
-      <c r="H4" s="72" t="s">
+      <c r="H4" s="77" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="72"/>
-      <c r="J4" s="72"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -2724,16 +2840,16 @@
       <c r="E6" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="G6" s="74" t="s">
+      <c r="G6" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="H6" s="74" t="s">
+      <c r="H6" s="54" t="s">
         <v>135</v>
       </c>
-      <c r="I6" s="74" t="s">
+      <c r="I6" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="J6" s="74" t="s">
+      <c r="J6" s="54" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2750,19 +2866,19 @@
       <c r="D7" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="E7" s="56" t="s">
+      <c r="E7" s="73" t="s">
         <v>111</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="G7" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="H7" s="75" t="s">
+      <c r="H7" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="I7" s="75" t="s">
+      <c r="I7" s="55" t="s">
         <v>176</v>
       </c>
-      <c r="J7" s="75" t="s">
+      <c r="J7" s="55" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2779,17 +2895,17 @@
       <c r="D8" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="G8" s="76" t="s">
+      <c r="E8" s="73"/>
+      <c r="G8" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="H8" s="77" t="s">
+      <c r="H8" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="I8" s="77" t="s">
+      <c r="I8" s="57" t="s">
         <v>140</v>
       </c>
-      <c r="J8" s="78">
+      <c r="J8" s="58">
         <v>255255255255</v>
       </c>
     </row>
@@ -2903,9 +3019,9 @@
       <c r="A6" t="s">
         <v>146</v>
       </c>
-      <c r="B6" s="76" t="str">
+      <c r="B6" s="56" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>331F017E</v>
+        <v>E04FF26F</v>
       </c>
       <c r="D6" t="s">
         <v>150</v>
@@ -2988,9 +3104,9 @@
       <c r="A13" t="s">
         <v>146</v>
       </c>
-      <c r="B13" s="76" t="str">
+      <c r="B13" s="56" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>95E82C30</v>
+        <v>33913338</v>
       </c>
       <c r="D13" t="s">
         <v>150</v>
@@ -3057,7 +3173,7 @@
     <col min="2" max="2" width="15.5703125" style="44" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3" customWidth="1"/>
     <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="82" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="60" customWidth="1"/>
     <col min="6" max="6" width="9.5703125" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5703125" style="10" bestFit="1" customWidth="1"/>
@@ -3077,18 +3193,18 @@
       <c r="D1" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="81" t="s">
+      <c r="E1" s="78" t="s">
         <v>184</v>
       </c>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81" t="s">
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78" t="s">
         <v>185</v>
       </c>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -3100,7 +3216,7 @@
       <c r="D2" t="s">
         <v>180</v>
       </c>
-      <c r="E2" s="82" t="s">
+      <c r="E2" s="60" t="s">
         <v>171</v>
       </c>
       <c r="F2" s="10" t="s">
@@ -3135,22 +3251,22 @@
       <c r="D3" t="s">
         <v>181</v>
       </c>
-      <c r="E3" s="82" t="s">
+      <c r="E3" s="60" t="s">
         <v>187</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="G3" s="84" t="s">
+      <c r="G3" s="61" t="s">
         <v>192</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="I3" s="82" t="s">
+      <c r="I3" s="60" t="s">
         <v>197</v>
       </c>
-      <c r="K3" s="84" t="s">
+      <c r="K3" s="61" t="s">
         <v>201</v>
       </c>
     </row>
@@ -3164,22 +3280,22 @@
       <c r="D4" t="s">
         <v>182</v>
       </c>
-      <c r="E4" s="82" t="s">
+      <c r="E4" s="60" t="s">
         <v>188</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="G4" s="84" t="s">
+      <c r="G4" s="61" t="s">
         <v>193</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="82" t="s">
+      <c r="I4" s="60" t="s">
         <v>198</v>
       </c>
-      <c r="K4" s="84" t="s">
+      <c r="K4" s="61" t="s">
         <v>202</v>
       </c>
     </row>
@@ -3193,22 +3309,22 @@
       <c r="D5" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="82" t="s">
+      <c r="E5" s="60" t="s">
         <v>189</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="G5" s="84" t="s">
+      <c r="G5" s="61" t="s">
         <v>194</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="I5" s="82" t="s">
+      <c r="I5" s="60" t="s">
         <v>199</v>
       </c>
-      <c r="K5" s="84" t="s">
+      <c r="K5" s="61" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3222,76 +3338,76 @@
       <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="82" t="s">
+      <c r="E6" s="60" t="s">
         <v>190</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="G6" s="84" t="s">
+      <c r="G6" s="61" t="s">
         <v>195</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="I6" s="81" t="s">
+      <c r="I6" s="78" t="s">
         <v>127</v>
       </c>
-      <c r="J6" s="81"/>
-      <c r="K6" s="81"/>
-      <c r="L6" s="81"/>
+      <c r="J6" s="78"/>
+      <c r="K6" s="78"/>
+      <c r="L6" s="78"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="79" t="str">
+      <c r="B7" s="59" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>D8258CFE</v>
+        <v>F217E85</v>
       </c>
       <c r="D7" t="s">
         <v>183</v>
       </c>
-      <c r="E7" s="82" t="s">
+      <c r="E7" s="60" t="s">
         <v>191</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="G7" s="84" t="s">
+      <c r="G7" s="61" t="s">
         <v>196</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="I7" s="81" t="s">
+      <c r="I7" s="78" t="s">
         <v>200</v>
       </c>
-      <c r="J7" s="81"/>
-      <c r="K7" s="81"/>
-      <c r="L7" s="81"/>
+      <c r="J7" s="78"/>
+      <c r="K7" s="78"/>
+      <c r="L7" s="78"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>186</v>
       </c>
-      <c r="E8" s="83">
+      <c r="E8" s="79">
         <f>2^32</f>
         <v>4294967296</v>
       </c>
-      <c r="F8" s="83"/>
-      <c r="G8" s="83"/>
-      <c r="H8" s="83"/>
-      <c r="I8" s="83">
+      <c r="F8" s="79"/>
+      <c r="G8" s="79"/>
+      <c r="H8" s="79"/>
+      <c r="I8" s="79">
         <f>2^32</f>
         <v>4294967296</v>
       </c>
-      <c r="J8" s="83"/>
-      <c r="K8" s="83"/>
-      <c r="L8" s="83"/>
+      <c r="J8" s="79"/>
+      <c r="K8" s="79"/>
+      <c r="L8" s="79"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="46" t="s">
         <v>155</v>
       </c>
       <c r="B9" s="14" t="s">
@@ -3299,52 +3415,52 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="B10" s="67" t="s">
+      <c r="B10" s="52" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+      <c r="A11" t="s">
         <v>158</v>
       </c>
-      <c r="B11" s="68">
+      <c r="B11" s="44">
         <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="59" t="s">
+      <c r="A12" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="B12" s="67" t="s">
+      <c r="B12" s="52" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="60" t="s">
+      <c r="A13" t="s">
         <v>159</v>
       </c>
-      <c r="B13" s="80" t="s">
+      <c r="B13" s="45" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="67" t="s">
+      <c r="B14" s="52" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="79" t="str">
+      <c r="B15" s="59" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>66D08586</v>
+        <v>84DC207E</v>
       </c>
     </row>
   </sheetData>
@@ -3378,333 +3494,333 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="65" t="s">
+      <c r="D1" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="E1" s="65" t="s">
+      <c r="E1" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="G1" s="58" t="s">
+      <c r="G1" s="46" t="s">
         <v>167</v>
       </c>
-      <c r="H1" s="58" t="s">
+      <c r="H1" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="I1" s="58" t="s">
+      <c r="I1" s="46" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="63">
+      <c r="B2" s="15">
         <v>49810</v>
       </c>
-      <c r="D2" s="63" t="s">
+      <c r="D2" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="63">
+      <c r="E2" s="15">
         <v>68</v>
       </c>
-      <c r="G2" s="63" t="s">
+      <c r="G2" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="H2" s="63">
+      <c r="H2" s="15">
         <v>0</v>
       </c>
-      <c r="I2" s="63">
+      <c r="I2" s="15">
         <v>1023</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="60">
+      <c r="B3">
         <v>22</v>
       </c>
-      <c r="D3" s="60" t="s">
+      <c r="D3" t="s">
         <v>163</v>
       </c>
-      <c r="E3" s="60">
+      <c r="E3">
         <v>67</v>
       </c>
-      <c r="G3" s="60" t="s">
+      <c r="G3" t="s">
         <v>169</v>
       </c>
-      <c r="H3" s="60">
+      <c r="H3">
         <v>1024</v>
       </c>
-      <c r="I3" s="60">
+      <c r="I3">
         <v>49151</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="59">
+      <c r="B4" s="18">
         <v>0</v>
       </c>
-      <c r="D4" s="59" t="s">
+      <c r="D4" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="59">
+      <c r="E4" s="18">
         <v>65535</v>
       </c>
-      <c r="G4" s="59" t="s">
+      <c r="G4" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="H4" s="59">
+      <c r="H4" s="18">
         <v>49152</v>
       </c>
-      <c r="I4" s="59">
+      <c r="I4" s="18">
         <v>65535</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="60" t="s">
+      <c r="A5" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="60">
+      <c r="B5">
         <v>0</v>
       </c>
-      <c r="D5" s="60" t="s">
+      <c r="D5" t="s">
         <v>160</v>
       </c>
       <c r="E5" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>F5FCFD96</v>
+        <v>11F498F2</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="59" t="s">
+      <c r="A6" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B6" s="59">
+      <c r="B6" s="18">
         <v>65535</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="47" t="s">
         <v>160</v>
       </c>
       <c r="B7" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>9272EBB7</v>
-      </c>
-      <c r="D7" s="65" t="s">
+        <v>8D5E980</v>
+      </c>
+      <c r="D7" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="E7" s="65" t="s">
+      <c r="E7" s="50" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D8" s="63" t="s">
+      <c r="D8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="E8" s="63">
+      <c r="E8" s="15">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="46" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="60" t="s">
+      <c r="D9" t="s">
         <v>163</v>
       </c>
-      <c r="E9" s="60">
+      <c r="E9">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="63">
+      <c r="B10" s="15">
         <v>22</v>
       </c>
-      <c r="D10" s="59" t="s">
+      <c r="D10" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="E10" s="59">
+      <c r="E10" s="18">
         <v>16384</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+      <c r="A11" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="60">
+      <c r="B11">
         <v>49810</v>
       </c>
-      <c r="D11" s="60" t="s">
+      <c r="D11" t="s">
         <v>160</v>
       </c>
       <c r="E11" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>5D15AE6D</v>
+        <v>1D274616</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="59" t="s">
+      <c r="A12" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B12" s="59">
+      <c r="B12" s="18">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="60" t="s">
+      <c r="A13" t="s">
         <v>165</v>
       </c>
-      <c r="B13" s="60">
+      <c r="B13">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B14" s="59">
+      <c r="B14" s="18">
         <v>16384</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="61" t="str">
+      <c r="B15" s="47" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>189999A6</v>
+        <v>4391332D</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="46" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="63" t="s">
+      <c r="A18" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="B18" s="63">
+      <c r="B18" s="15">
         <v>49810</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="60" t="s">
+      <c r="A19" t="s">
         <v>163</v>
       </c>
-      <c r="B19" s="60">
+      <c r="B19">
         <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="59" t="s">
+      <c r="A20" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B20" s="59">
+      <c r="B20" s="18">
         <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="60" t="s">
+      <c r="A21" t="s">
         <v>165</v>
       </c>
-      <c r="B21" s="60">
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="59" t="s">
+      <c r="A22" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B22" s="59">
+      <c r="B22" s="18">
         <v>16384</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="61" t="s">
+      <c r="A23" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="B23" s="61" t="str">
+      <c r="B23" s="47" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>1F3E77C1</v>
+        <v>56A363E9</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="58" t="s">
+      <c r="A25" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="46" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="B26" s="63">
+      <c r="B26" s="15">
         <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="60" t="s">
+      <c r="A27" t="s">
         <v>163</v>
       </c>
-      <c r="B27" s="60">
+      <c r="B27">
         <v>49810</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B28" s="59">
+      <c r="B28" s="18">
         <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="60" t="s">
+      <c r="A29" t="s">
         <v>165</v>
       </c>
-      <c r="B29" s="60">
+      <c r="B29">
         <v>300</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="59" t="s">
+      <c r="A30" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B30" s="59">
+      <c r="B30" s="18">
         <v>16384</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="B31" s="61" t="str">
+      <c r="B31" s="47" t="str">
         <f ca="1">DEC2HEX((RAND()*2^32))</f>
-        <v>A7CAFF7E</v>
+        <v>40DFD659</v>
       </c>
     </row>
   </sheetData>
@@ -3724,4 +3840,299 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D30B036F-4FE9-4BFD-A02A-77D3A20270F2}">
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D1" t="s">
+        <v>217</v>
+      </c>
+      <c r="F1" t="s">
+        <v>252</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="H1" t="s">
+        <v>218</v>
+      </c>
+      <c r="K1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="I2" s="80" t="s">
+        <v>236</v>
+      </c>
+      <c r="K2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>245</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="I3" s="80" t="s">
+        <v>237</v>
+      </c>
+      <c r="K3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>246</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="I4" s="80" t="s">
+        <v>238</v>
+      </c>
+      <c r="K4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>247</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="I5" s="80" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>248</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="I6" s="80" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="I7" s="80" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>250</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="I8" s="80" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>7</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="F9" t="s">
+        <v>251</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="I9" s="80" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D13" s="44" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D14" s="44" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D15" s="44" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D16" s="44" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="44" t="s">
+        <v>219</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>